<commit_message>
first step of event-recognition dataset prep
</commit_message>
<xml_diff>
--- a/processed/airdata/correction_log_step_3.xlsx
+++ b/processed/airdata/correction_log_step_3.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Data Kuliah\Semester 8\IEEE - TIFS\dataset-tool\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Data Kuliah\Semester 8\IEEE - TIFS\dataset\processed\airdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D35B114F-7011-4DC3-ACFC-A40536D8CCF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDF36611-0F8F-4C5E-B22E-4F82C87EF803}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" xr2:uid="{2C9B559C-DB3E-4A5F-A7EF-9A6DED2CF13B}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="45">
   <si>
     <t>MessageID</t>
   </si>
@@ -168,6 +168,9 @@
   </si>
   <si>
     <t>Likely scenario: Propeller Failure. Missing front propeller causes rear pitch (no collision).</t>
+  </si>
+  <si>
+    <t>ambiguous patterns, too much abstraction</t>
   </si>
 </sst>
 </file>
@@ -203,9 +206,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -540,7 +542,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A2728F41-E64C-41D0-B04E-388C9EF5B89E}">
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:D26"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.28515625" customWidth="1"/>
@@ -570,7 +572,7 @@
       <c r="B2" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" t="s">
         <v>34</v>
       </c>
       <c r="D2" t="s">
@@ -584,7 +586,7 @@
       <c r="B3" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" t="s">
         <v>36</v>
       </c>
       <c r="D3" t="s">
@@ -598,7 +600,7 @@
       <c r="B4" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" t="s">
         <v>38</v>
       </c>
       <c r="D4" t="s">
@@ -612,7 +614,7 @@
       <c r="B5" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" t="s">
         <v>40</v>
       </c>
       <c r="D5" t="s">
@@ -626,7 +628,7 @@
       <c r="B6" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" t="s">
         <v>42</v>
       </c>
       <c r="D6" t="s">
@@ -640,7 +642,7 @@
       <c r="B7" t="s">
         <v>6</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="C7" t="s">
         <v>7</v>
       </c>
       <c r="D7" t="s">
@@ -654,7 +656,7 @@
       <c r="B8" t="s">
         <v>6</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="C8" t="s">
         <v>8</v>
       </c>
       <c r="D8" t="s">
@@ -668,7 +670,7 @@
       <c r="B9" t="s">
         <v>6</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="C9" t="s">
         <v>9</v>
       </c>
       <c r="D9" t="s">
@@ -682,7 +684,7 @@
       <c r="B10" t="s">
         <v>6</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="C10" t="s">
         <v>10</v>
       </c>
       <c r="D10" t="s">
@@ -897,6 +899,20 @@
       </c>
       <c r="D25" t="s">
         <v>32</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>484</v>
+      </c>
+      <c r="B26" t="s">
+        <v>30</v>
+      </c>
+      <c r="C26" t="s">
+        <v>31</v>
+      </c>
+      <c r="D26" t="s">
+        <v>44</v>
       </c>
     </row>
   </sheetData>

</xml_diff>